<commit_message>
Add 6mm straight and elbow push-in fittings for brass and stainless steel, renumber database 1099.1000 to 1099.1069, update Excel and selector options
</commit_message>
<xml_diff>
--- a/backup database/odoo_koppelingen_import_v2.xlsx
+++ b/backup database/odoo_koppelingen_import_v2.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G64"/>
+  <dimension ref="A1:G72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -1531,12 +1531,12 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Rechte insteekkoppeling 8 mm - G 1/8" M (Messing vernikkeld)</t>
+          <t>Rechte insteekkoppeling 6 mm - G 1/8" M (Messing vernikkeld)</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Push-in 8 mm</t>
+          <t>Push-in 6 mm</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1551,12 +1551,12 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Insteekkoppelingen 8 mm</t>
+          <t>Insteekkoppelingen 6 mm</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Rechte steekkoppeling voor 8 mm leiding x G 1/8" buitendraad (Messing vernikkeld)</t>
+          <t>Rechte steekkoppeling voor 6 mm leiding x G 1/8" buitendraad (Messing vernikkeld)</t>
         </is>
       </c>
     </row>
@@ -1568,12 +1568,12 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Knie-insteekkoppeling 90° 8 mm - G 1/8" M (Messing vernikkeld)</t>
+          <t>Knie-insteekkoppeling 90° 6 mm - G 1/8" M (Messing vernikkeld)</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Push-in 8 mm</t>
+          <t>Push-in 6 mm</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1588,12 +1588,12 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Insteekkoppelingen 8 mm</t>
+          <t>Insteekkoppelingen 6 mm</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>90° haakse knie-steekkoppeling voor 8 mm leiding x G 1/8" buitendraad (Messing vernikkeld)</t>
+          <t>90° haakse knie-steekkoppeling voor 6 mm leiding x G 1/8" buitendraad (Messing vernikkeld)</t>
         </is>
       </c>
     </row>
@@ -1605,12 +1605,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Rechte insteekkoppeling 8 mm - G 1/4" M (Messing vernikkeld)</t>
+          <t>Rechte insteekkoppeling 6 mm - G 1/4" M (Messing vernikkeld)</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Push-in 8 mm</t>
+          <t>Push-in 6 mm</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1625,12 +1625,12 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Insteekkoppelingen 8 mm</t>
+          <t>Insteekkoppelingen 6 mm</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Rechte steekkoppeling voor 8 mm leiding x G 1/4" buitendraad (Messing vernikkeld)</t>
+          <t>Rechte steekkoppeling voor 6 mm leiding x G 1/4" buitendraad (Messing vernikkeld)</t>
         </is>
       </c>
     </row>
@@ -1642,12 +1642,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Knie-insteekkoppeling 90° 8 mm - G 1/4" M (Messing vernikkeld)</t>
+          <t>Knie-insteekkoppeling 90° 6 mm - G 1/4" M (Messing vernikkeld)</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Push-in 8 mm</t>
+          <t>Push-in 6 mm</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1662,12 +1662,12 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Insteekkoppelingen 8 mm</t>
+          <t>Insteekkoppelingen 6 mm</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>90° haakse knie-steekkoppeling voor 8 mm leiding x G 1/4" buitendraad (Messing vernikkeld)</t>
+          <t>90° haakse knie-steekkoppeling voor 6 mm leiding x G 1/4" buitendraad (Messing vernikkeld)</t>
         </is>
       </c>
     </row>
@@ -1679,32 +1679,32 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Verloopstuk M6x1 M x G 1/4" F (RVS)</t>
+          <t>Rechte insteekkoppeling 8 mm - G 1/8" M (Messing vernikkeld)</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>M6x1 M (buitendraad recht)</t>
+          <t>Push-in 8 mm</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>G 1/4" F (binnendraad)</t>
+          <t>G 1/8" BSPP M (buitendraad recht)</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>RVS</t>
+          <t>Messing vernikkeld</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Verloopstukken naar G 1/4"</t>
+          <t>Insteekkoppelingen 8 mm</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Draadadapter buitendraad M6x1 naar binnendraad G 1/4" BSPP (RVS)</t>
+          <t>Rechte steekkoppeling voor 8 mm leiding x G 1/8" buitendraad (Messing vernikkeld)</t>
         </is>
       </c>
     </row>
@@ -1716,32 +1716,32 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Verloopstuk M8x1 M x G 1/4" F (RVS)</t>
+          <t>Knie-insteekkoppeling 90° 8 mm - G 1/8" M (Messing vernikkeld)</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>M8x1 M (buitendraad recht)</t>
+          <t>Push-in 8 mm</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>G 1/4" F (binnendraad)</t>
+          <t>G 1/8" BSPP M (90° knie recht)</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>RVS</t>
+          <t>Messing vernikkeld</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Verloopstukken naar G 1/4"</t>
+          <t>Insteekkoppelingen 8 mm</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Draadadapter buitendraad M8x1 naar binnendraad G 1/4" BSPP (RVS)</t>
+          <t>90° haakse knie-steekkoppeling voor 8 mm leiding x G 1/8" buitendraad (Messing vernikkeld)</t>
         </is>
       </c>
     </row>
@@ -1753,32 +1753,32 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Verloopstuk M8x1.25 M x G 1/4" F (RVS)</t>
+          <t>Rechte insteekkoppeling 8 mm - G 1/4" M (Messing vernikkeld)</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>M8x1.25 M (buitendraad recht)</t>
+          <t>Push-in 8 mm</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>G 1/4" F (binnendraad)</t>
+          <t>G 1/4" BSPP M (buitendraad recht)</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>RVS</t>
+          <t>Messing vernikkeld</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Verloopstukken naar G 1/4"</t>
+          <t>Insteekkoppelingen 8 mm</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Draadadapter buitendraad M8x1.25 naar binnendraad G 1/4" BSPP (RVS)</t>
+          <t>Rechte steekkoppeling voor 8 mm leiding x G 1/4" buitendraad (Messing vernikkeld)</t>
         </is>
       </c>
     </row>
@@ -1790,32 +1790,32 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Verloopstuk M10x1 M x G 1/4" F (RVS)</t>
+          <t>Knie-insteekkoppeling 90° 8 mm - G 1/4" M (Messing vernikkeld)</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>M10x1 M (buitendraad recht)</t>
+          <t>Push-in 8 mm</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>G 1/4" F (binnendraad)</t>
+          <t>G 1/4" BSPP M (90° knie recht)</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>RVS</t>
+          <t>Messing vernikkeld</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Verloopstukken naar G 1/4"</t>
+          <t>Insteekkoppelingen 8 mm</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Draadadapter buitendraad M10x1 naar binnendraad G 1/4" BSPP (RVS)</t>
+          <t>90° haakse knie-steekkoppeling voor 8 mm leiding x G 1/4" buitendraad (Messing vernikkeld)</t>
         </is>
       </c>
     </row>
@@ -1827,12 +1827,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Verloopstuk M10x1.5 M x G 1/4" F (RVS)</t>
+          <t>Verloopstuk M6x1 M x G 1/4" F (RVS)</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>M10x1.5 M (buitendraad recht)</t>
+          <t>M6x1 M (buitendraad recht)</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -1852,7 +1852,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Draadadapter buitendraad M10x1.5 naar binnendraad G 1/4" BSPP (RVS)</t>
+          <t>Draadadapter buitendraad M6x1 naar binnendraad G 1/4" BSPP (RVS)</t>
         </is>
       </c>
     </row>
@@ -1864,12 +1864,12 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Verloopstuk G 1/8 M x G 1/4" F (RVS)</t>
+          <t>Verloopstuk M8x1 M x G 1/4" F (RVS)</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>G 1/8" M (buitendraad)</t>
+          <t>M8x1 M (buitendraad recht)</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1889,7 +1889,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Draadadapter buitendraad G 1/8 naar binnendraad G 1/4" BSPP (RVS)</t>
+          <t>Draadadapter buitendraad M8x1 naar binnendraad G 1/4" BSPP (RVS)</t>
         </is>
       </c>
     </row>
@@ -1901,12 +1901,12 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Verloopstuk 1/8 NPT M x G 1/4" F (RVS)</t>
+          <t>Verloopstuk M8x1.25 M x G 1/4" F (RVS)</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>1/8" NPT M (buitendraad conisch)</t>
+          <t>M8x1.25 M (buitendraad recht)</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -1926,7 +1926,7 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Draadadapter buitendraad 1/8 NPT naar binnendraad G 1/4" BSPP (RVS)</t>
+          <t>Draadadapter buitendraad M8x1.25 naar binnendraad G 1/4" BSPP (RVS)</t>
         </is>
       </c>
     </row>
@@ -1938,12 +1938,12 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Verloopstuk 1/4 NPT M x G 1/4" F (RVS)</t>
+          <t>Verloopstuk M10x1 M x G 1/4" F (RVS)</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>1/4" NPT M (buitendraad conisch)</t>
+          <t>M10x1 M (buitendraad recht)</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -1963,7 +1963,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Draadadapter buitendraad 1/4 NPT naar binnendraad G 1/4" BSPP (RVS)</t>
+          <t>Draadadapter buitendraad M10x1 naar binnendraad G 1/4" BSPP (RVS)</t>
         </is>
       </c>
     </row>
@@ -1975,17 +1975,17 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Verloopstuk M6x1 M x G 1/8" F (RVS)</t>
+          <t>Verloopstuk M10x1.5 M x G 1/4" F (RVS)</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>M6x1 M (buitendraad recht)</t>
+          <t>M10x1.5 M (buitendraad recht)</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>G 1/8" F (binnendraad)</t>
+          <t>G 1/4" F (binnendraad)</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -1995,12 +1995,12 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Verloopstukken naar G 1/8"</t>
+          <t>Verloopstukken naar G 1/4"</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Draadadapter buitendraad M6x1 naar binnendraad G 1/8" BSPP (RVS)</t>
+          <t>Draadadapter buitendraad M10x1.5 naar binnendraad G 1/4" BSPP (RVS)</t>
         </is>
       </c>
     </row>
@@ -2012,17 +2012,17 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Verloopstuk M8x1 M x G 1/8" F (RVS)</t>
+          <t>Verloopstuk G 1/8 M x G 1/4" F (RVS)</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>M8x1 M (buitendraad recht)</t>
+          <t>G 1/8" M (buitendraad)</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>G 1/8" F (binnendraad)</t>
+          <t>G 1/4" F (binnendraad)</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -2032,12 +2032,12 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Verloopstukken naar G 1/8"</t>
+          <t>Verloopstukken naar G 1/4"</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Draadadapter buitendraad M8x1 naar binnendraad G 1/8" BSPP (RVS)</t>
+          <t>Draadadapter buitendraad G 1/8 naar binnendraad G 1/4" BSPP (RVS)</t>
         </is>
       </c>
     </row>
@@ -2049,17 +2049,17 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Verloopstuk M8x1.25 M x G 1/8" F (RVS)</t>
+          <t>Verloopstuk 1/8 NPT M x G 1/4" F (RVS)</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>M8x1.25 M (buitendraad recht)</t>
+          <t>1/8" NPT M (buitendraad conisch)</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>G 1/8" F (binnendraad)</t>
+          <t>G 1/4" F (binnendraad)</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -2069,12 +2069,12 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Verloopstukken naar G 1/8"</t>
+          <t>Verloopstukken naar G 1/4"</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Draadadapter buitendraad M8x1.25 naar binnendraad G 1/8" BSPP (RVS)</t>
+          <t>Draadadapter buitendraad 1/8 NPT naar binnendraad G 1/4" BSPP (RVS)</t>
         </is>
       </c>
     </row>
@@ -2086,17 +2086,17 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Verloopstuk M10x1 M x G 1/8" F (RVS)</t>
+          <t>Verloopstuk 1/4 NPT M x G 1/4" F (RVS)</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>M10x1 M (buitendraad recht)</t>
+          <t>1/4" NPT M (buitendraad conisch)</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>G 1/8" F (binnendraad)</t>
+          <t>G 1/4" F (binnendraad)</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -2106,12 +2106,12 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Verloopstukken naar G 1/8"</t>
+          <t>Verloopstukken naar G 1/4"</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Draadadapter buitendraad M10x1 naar binnendraad G 1/8" BSPP (RVS)</t>
+          <t>Draadadapter buitendraad 1/4 NPT naar binnendraad G 1/4" BSPP (RVS)</t>
         </is>
       </c>
     </row>
@@ -2123,12 +2123,12 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Verloopstuk G 1/4 M x G 1/8" F (RVS)</t>
+          <t>Verloopstuk M6x1 M x G 1/8" F (RVS)</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>G 1/4" M (buitendraad)</t>
+          <t>M6x1 M (buitendraad recht)</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -2148,7 +2148,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Draadadapter buitendraad G 1/4 naar binnendraad G 1/8" BSPP (RVS)</t>
+          <t>Draadadapter buitendraad M6x1 naar binnendraad G 1/8" BSPP (RVS)</t>
         </is>
       </c>
     </row>
@@ -2160,12 +2160,12 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Verloopstuk 1/8 NPT M x G 1/8" F (RVS)</t>
+          <t>Verloopstuk M8x1 M x G 1/8" F (RVS)</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>1/8" NPT M (buitendraad conisch)</t>
+          <t>M8x1 M (buitendraad recht)</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -2185,7 +2185,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Draadadapter buitendraad 1/8 NPT naar binnendraad G 1/8" BSPP (RVS)</t>
+          <t>Draadadapter buitendraad M8x1 naar binnendraad G 1/8" BSPP (RVS)</t>
         </is>
       </c>
     </row>
@@ -2197,17 +2197,17 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Verloopstuk G 1/8" M x G 1/4" F (RVS)</t>
+          <t>Verloopstuk M8x1.25 M x G 1/8" F (RVS)</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>G 1/8" M (buitendraad)</t>
+          <t>M8x1.25 M (buitendraad recht)</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>G 1/4" F (binnendraad)</t>
+          <t>G 1/8" F (binnendraad)</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -2217,12 +2217,12 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Verloopstukken</t>
+          <t>Verloopstukken naar G 1/8"</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Verloopadapter van G 1/8" buitendraad naar G 1/4" binnendraad voor ISPL (RVS)</t>
+          <t>Draadadapter buitendraad M8x1.25 naar binnendraad G 1/8" BSPP (RVS)</t>
         </is>
       </c>
     </row>
@@ -2234,17 +2234,17 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Kniestuk 90° G 1/4" M x G 1/4" F (RVS)</t>
+          <t>Verloopstuk M10x1 M x G 1/8" F (RVS)</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>G 1/4" M (buitendraad)</t>
+          <t>M10x1 M (buitendraad recht)</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>G 1/4" F (binnendraad 90°)</t>
+          <t>G 1/8" F (binnendraad)</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -2254,12 +2254,12 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Kniestukken G 1/4"</t>
+          <t>Verloopstukken naar G 1/8"</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Haakse koppeling 90° buitendraad G 1/4" naar binnendraad G 1/4" (RVS)</t>
+          <t>Draadadapter buitendraad M10x1 naar binnendraad G 1/8" BSPP (RVS)</t>
         </is>
       </c>
     </row>
@@ -2271,7 +2271,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Kniestuk 45° G 1/4" M x G 1/4" F (RVS)</t>
+          <t>Verloopstuk G 1/4 M x G 1/8" F (RVS)</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2281,7 +2281,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>G 1/4" F (binnendraad 45°)</t>
+          <t>G 1/8" F (binnendraad)</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -2291,12 +2291,12 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Kniestukken G 1/4"</t>
+          <t>Verloopstukken naar G 1/8"</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>Kniestuk 45° buitendraad G 1/4" naar binnendraad G 1/4" (RVS)</t>
+          <t>Draadadapter buitendraad G 1/4 naar binnendraad G 1/8" BSPP (RVS)</t>
         </is>
       </c>
     </row>
@@ -2308,17 +2308,17 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Kniestuk 90° G 1/8" M x G 1/8" F (RVS)</t>
+          <t>Verloopstuk 1/8 NPT M x G 1/8" F (RVS)</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>G 1/8" M (buitendraad)</t>
+          <t>1/8" NPT M (buitendraad conisch)</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>G 1/8" F (binnendraad 90°)</t>
+          <t>G 1/8" F (binnendraad)</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -2328,12 +2328,12 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Kniestukken G 1/8"</t>
+          <t>Verloopstukken naar G 1/8"</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Haakse koppeling 90° buitendraad G 1/8" naar binnendraad G 1/8" (RVS)</t>
+          <t>Draadadapter buitendraad 1/8 NPT naar binnendraad G 1/8" BSPP (RVS)</t>
         </is>
       </c>
     </row>
@@ -2345,7 +2345,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Kniestuk 45° G 1/8" M x G 1/8" F (RVS)</t>
+          <t>Verloopstuk G 1/8" M x G 1/4" F (RVS)</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2355,7 +2355,7 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>G 1/8" F (binnendraad 45°)</t>
+          <t>G 1/4" F (binnendraad)</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -2365,12 +2365,12 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Kniestukken G 1/8"</t>
+          <t>Verloopstukken</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Kniestuk 45° buitendraad G 1/8" naar binnendraad G 1/8" (RVS)</t>
+          <t>Verloopadapter van G 1/8" buitendraad naar G 1/4" binnendraad voor ISPL (RVS)</t>
         </is>
       </c>
     </row>
@@ -2382,7 +2382,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Verlengstuk G 1/4" M x G 1/4" F - L=15mm (RVS)</t>
+          <t>Kniestuk 90° G 1/4" M x G 1/4" F (RVS)</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2392,7 +2392,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>G 1/4" F (binnendraad) - L=15mm</t>
+          <t>G 1/4" F (binnendraad 90°)</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -2402,12 +2402,12 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Verlengstukken G 1/4"</t>
+          <t>Kniestukken G 1/4"</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>Verlengstuk buitendraad G 1/4" naar binnendraad G 1/4", effectieve lengte 15 mm (RVS)</t>
+          <t>Haakse koppeling 90° buitendraad G 1/4" naar binnendraad G 1/4" (RVS)</t>
         </is>
       </c>
     </row>
@@ -2419,17 +2419,17 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Verlengstuk G 1/8" M x G 1/8" F - L=15mm (RVS)</t>
+          <t>Kniestuk 45° G 1/4" M x G 1/4" F (RVS)</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>G 1/8" M (buitendraad)</t>
+          <t>G 1/4" M (buitendraad)</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>G 1/8" F (binnendraad) - L=15mm</t>
+          <t>G 1/4" F (binnendraad 45°)</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -2439,12 +2439,12 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Verlengstukken G 1/8"</t>
+          <t>Kniestukken G 1/4"</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>Verlengstuk buitendraad G 1/8" naar binnendraad G 1/8", effectieve lengte 15 mm (RVS)</t>
+          <t>Kniestuk 45° buitendraad G 1/4" naar binnendraad G 1/4" (RVS)</t>
         </is>
       </c>
     </row>
@@ -2456,17 +2456,17 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Verlengstuk G 1/4" M x G 1/4" F - L=25mm (RVS)</t>
+          <t>Kniestuk 90° G 1/8" M x G 1/8" F (RVS)</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>G 1/4" M (buitendraad)</t>
+          <t>G 1/8" M (buitendraad)</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>G 1/4" F (binnendraad) - L=25mm</t>
+          <t>G 1/8" F (binnendraad 90°)</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -2476,12 +2476,12 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Verlengstukken G 1/4"</t>
+          <t>Kniestukken G 1/8"</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>Verlengstuk buitendraad G 1/4" naar binnendraad G 1/4", effectieve lengte 25 mm (RVS)</t>
+          <t>Haakse koppeling 90° buitendraad G 1/8" naar binnendraad G 1/8" (RVS)</t>
         </is>
       </c>
     </row>
@@ -2493,7 +2493,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Verlengstuk G 1/8" M x G 1/8" F - L=25mm (RVS)</t>
+          <t>Kniestuk 45° G 1/8" M x G 1/8" F (RVS)</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -2503,7 +2503,7 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>G 1/8" F (binnendraad) - L=25mm</t>
+          <t>G 1/8" F (binnendraad 45°)</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -2513,12 +2513,12 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Verlengstukken G 1/8"</t>
+          <t>Kniestukken G 1/8"</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>Verlengstuk buitendraad G 1/8" naar binnendraad G 1/8", effectieve lengte 25 mm (RVS)</t>
+          <t>Kniestuk 45° buitendraad G 1/8" naar binnendraad G 1/8" (RVS)</t>
         </is>
       </c>
     </row>
@@ -2530,7 +2530,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Verlengstuk G 1/4" M x G 1/4" F - L=35mm (RVS)</t>
+          <t>Verlengstuk G 1/4" M x G 1/4" F - L=15mm (RVS)</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -2540,7 +2540,7 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>G 1/4" F (binnendraad) - L=35mm</t>
+          <t>G 1/4" F (binnendraad) - L=15mm</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -2555,7 +2555,7 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>Verlengstuk buitendraad G 1/4" naar binnendraad G 1/4", effectieve lengte 35 mm (RVS)</t>
+          <t>Verlengstuk buitendraad G 1/4" naar binnendraad G 1/4", effectieve lengte 15 mm (RVS)</t>
         </is>
       </c>
     </row>
@@ -2567,7 +2567,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Verlengstuk G 1/8" M x G 1/8" F - L=35mm (RVS)</t>
+          <t>Verlengstuk G 1/8" M x G 1/8" F - L=15mm (RVS)</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -2577,7 +2577,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>G 1/8" F (binnendraad) - L=35mm</t>
+          <t>G 1/8" F (binnendraad) - L=15mm</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -2592,7 +2592,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>Verlengstuk buitendraad G 1/8" naar binnendraad G 1/8", effectieve lengte 35 mm (RVS)</t>
+          <t>Verlengstuk buitendraad G 1/8" naar binnendraad G 1/8", effectieve lengte 15 mm (RVS)</t>
         </is>
       </c>
     </row>
@@ -2604,7 +2604,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Verlengstuk G 1/4" M x G 1/4" F - L=50mm (RVS)</t>
+          <t>Verlengstuk G 1/4" M x G 1/4" F - L=25mm (RVS)</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -2614,7 +2614,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>G 1/4" F (binnendraad) - L=50mm</t>
+          <t>G 1/4" F (binnendraad) - L=25mm</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -2629,7 +2629,7 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>Verlengstuk buitendraad G 1/4" naar binnendraad G 1/4", effectieve lengte 50 mm (RVS)</t>
+          <t>Verlengstuk buitendraad G 1/4" naar binnendraad G 1/4", effectieve lengte 25 mm (RVS)</t>
         </is>
       </c>
     </row>
@@ -2641,7 +2641,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Verlengstuk G 1/8" M x G 1/8" F - L=50mm (RVS)</t>
+          <t>Verlengstuk G 1/8" M x G 1/8" F - L=25mm (RVS)</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -2651,7 +2651,7 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>G 1/8" F (binnendraad) - L=50mm</t>
+          <t>G 1/8" F (binnendraad) - L=25mm</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -2666,7 +2666,7 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>Verlengstuk buitendraad G 1/8" naar binnendraad G 1/8", effectieve lengte 50 mm (RVS)</t>
+          <t>Verlengstuk buitendraad G 1/8" naar binnendraad G 1/8", effectieve lengte 25 mm (RVS)</t>
         </is>
       </c>
     </row>
@@ -2678,17 +2678,17 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Rechte insteekkoppeling 8 mm - G 1/8" M (RVS)</t>
+          <t>Verlengstuk G 1/4" M x G 1/4" F - L=35mm (RVS)</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Push-in 8 mm</t>
+          <t>G 1/4" M (buitendraad)</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>G 1/8" BSPP M (buitendraad recht)</t>
+          <t>G 1/4" F (binnendraad) - L=35mm</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -2698,12 +2698,12 @@
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Insteekkoppelingen 8 mm</t>
+          <t>Verlengstukken G 1/4"</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>Rechte steekkoppeling voor 8 mm leiding x G 1/8" buitendraad (RVS)</t>
+          <t>Verlengstuk buitendraad G 1/4" naar binnendraad G 1/4", effectieve lengte 35 mm (RVS)</t>
         </is>
       </c>
     </row>
@@ -2715,17 +2715,17 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Knie-insteekkoppeling 90° 8 mm - G 1/8" M (RVS)</t>
+          <t>Verlengstuk G 1/8" M x G 1/8" F - L=35mm (RVS)</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Push-in 8 mm</t>
+          <t>G 1/8" M (buitendraad)</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>G 1/8" BSPP M (90° knie recht)</t>
+          <t>G 1/8" F (binnendraad) - L=35mm</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -2735,12 +2735,12 @@
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>Insteekkoppelingen 8 mm</t>
+          <t>Verlengstukken G 1/8"</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>90° haakse knie-steekkoppeling voor 8 mm leiding x G 1/8" buitendraad (RVS)</t>
+          <t>Verlengstuk buitendraad G 1/8" naar binnendraad G 1/8", effectieve lengte 35 mm (RVS)</t>
         </is>
       </c>
     </row>
@@ -2752,17 +2752,17 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Rechte insteekkoppeling 8 mm - G 1/4" M (RVS)</t>
+          <t>Verlengstuk G 1/4" M x G 1/4" F - L=50mm (RVS)</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Push-in 8 mm</t>
+          <t>G 1/4" M (buitendraad)</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>G 1/4" BSPP M (buitendraad recht)</t>
+          <t>G 1/4" F (binnendraad) - L=50mm</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -2772,12 +2772,12 @@
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Insteekkoppelingen 8 mm</t>
+          <t>Verlengstukken G 1/4"</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>Rechte steekkoppeling voor 8 mm leiding x G 1/4" buitendraad (RVS)</t>
+          <t>Verlengstuk buitendraad G 1/4" naar binnendraad G 1/4", effectieve lengte 50 mm (RVS)</t>
         </is>
       </c>
     </row>
@@ -2789,30 +2789,326 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
+          <t>Verlengstuk G 1/8" M x G 1/8" F - L=50mm (RVS)</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>G 1/8" M (buitendraad)</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>G 1/8" F (binnendraad) - L=50mm</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>RVS</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>Verlengstukken G 1/8"</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>Verlengstuk buitendraad G 1/8" naar binnendraad G 1/8", effectieve lengte 50 mm (RVS)</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>1099.1062</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Rechte insteekkoppeling 6 mm - G 1/8" M (RVS)</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Push-in 6 mm</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>G 1/8" BSPP M (buitendraad recht)</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>RVS</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>Insteekkoppelingen 6 mm</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>Rechte steekkoppeling voor 6 mm leiding x G 1/8" buitendraad (RVS)</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>1099.1063</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Knie-insteekkoppeling 90° 6 mm - G 1/8" M (RVS)</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Push-in 6 mm</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>G 1/8" BSPP M (90° knie recht)</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>RVS</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>Insteekkoppelingen 6 mm</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>90° haakse knie-steekkoppeling voor 6 mm leiding x G 1/8" buitendraad (RVS)</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>1099.1064</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Rechte insteekkoppeling 6 mm - G 1/4" M (RVS)</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Push-in 6 mm</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>G 1/4" BSPP M (buitendraad recht)</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>RVS</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>Insteekkoppelingen 6 mm</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>Rechte steekkoppeling voor 6 mm leiding x G 1/4" buitendraad (RVS)</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>1099.1065</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Knie-insteekkoppeling 90° 6 mm - G 1/4" M (RVS)</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Push-in 6 mm</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>G 1/4" BSPP M (90° knie recht)</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>RVS</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>Insteekkoppelingen 6 mm</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>90° haakse knie-steekkoppeling voor 6 mm leiding x G 1/4" buitendraad (RVS)</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>1099.1066</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Rechte insteekkoppeling 8 mm - G 1/8" M (RVS)</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Push-in 8 mm</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>G 1/8" BSPP M (buitendraad recht)</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>RVS</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>Insteekkoppelingen 8 mm</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>Rechte steekkoppeling voor 8 mm leiding x G 1/8" buitendraad (RVS)</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>1099.1067</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Knie-insteekkoppeling 90° 8 mm - G 1/8" M (RVS)</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Push-in 8 mm</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>G 1/8" BSPP M (90° knie recht)</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>RVS</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>Insteekkoppelingen 8 mm</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>90° haakse knie-steekkoppeling voor 8 mm leiding x G 1/8" buitendraad (RVS)</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>1099.1068</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Rechte insteekkoppeling 8 mm - G 1/4" M (RVS)</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Push-in 8 mm</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>G 1/4" BSPP M (buitendraad recht)</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>RVS</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>Insteekkoppelingen 8 mm</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>Rechte steekkoppeling voor 8 mm leiding x G 1/4" buitendraad (RVS)</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>1099.1069</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
           <t>Knie-insteekkoppeling 90° 8 mm - G 1/4" M (RVS)</t>
         </is>
       </c>
-      <c r="C64" t="inlineStr">
+      <c r="C72" t="inlineStr">
         <is>
           <t>Push-in 8 mm</t>
         </is>
       </c>
-      <c r="D64" t="inlineStr">
+      <c r="D72" t="inlineStr">
         <is>
           <t>G 1/4" BSPP M (90° knie recht)</t>
         </is>
       </c>
-      <c r="E64" t="inlineStr">
+      <c r="E72" t="inlineStr">
         <is>
           <t>RVS</t>
         </is>
       </c>
-      <c r="F64" t="inlineStr">
+      <c r="F72" t="inlineStr">
         <is>
           <t>Insteekkoppelingen 8 mm</t>
         </is>
       </c>
-      <c r="G64" t="inlineStr">
+      <c r="G72" t="inlineStr">
         <is>
           <t>90° haakse knie-steekkoppeling voor 8 mm leiding x G 1/4" buitendraad (RVS)</t>
         </is>

</xml_diff>